<commit_message>
Updates for HMTM 2022 to pass
</commit_message>
<xml_diff>
--- a/data-raw/SAA.xlsx
+++ b/data-raw/SAA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11211"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebsilas/MST/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebsilas/SAA/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFB6E13D-9FB0-D448-ADF9-9FBECA5AA36B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A64825A3-D437-2347-BA27-260D9603B20C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1060" windowWidth="35840" windowHeight="19200" xr2:uid="{F918617E-B214-614F-96D8-792A3F23E788}"/>
+    <workbookView xWindow="1280" yWindow="2060" windowWidth="35840" windowHeight="19200" xr2:uid="{F918617E-B214-614F-96D8-792A3F23E788}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,9 +44,6 @@
     <t>en</t>
   </si>
   <si>
-    <t>Welcome to the Melody Singing Task!</t>
-  </si>
-  <si>
     <t>When you click the Play button in the next set of trials, you will hear a 5-second note</t>
   </si>
   <si>
@@ -62,18 +59,12 @@
     <t>How to Sing</t>
   </si>
   <si>
-    <t>mst_welcome</t>
-  </si>
-  <si>
     <t>long_tone_instruction</t>
   </si>
   <si>
     <t>long_tone_instruction_2</t>
   </si>
   <si>
-    <t>mst_button_play_note_and_sing</t>
-  </si>
-  <si>
     <t>After hearing the melody, do your best to sing it back, then click Stop. You can try each melody up to 3 times. It's okay if you don't think you got it, just try your best!</t>
   </si>
   <si>
@@ -86,30 +77,9 @@
     <t>sing_melody_trial_instructions3</t>
   </si>
   <si>
-    <t>mst_welcome_1</t>
-  </si>
-  <si>
-    <t>mst_welcome_2</t>
-  </si>
-  <si>
-    <t>mst_instructions1</t>
-  </si>
-  <si>
-    <t>mst_instructions2</t>
-  </si>
-  <si>
-    <t>mst_instructions3</t>
-  </si>
-  <si>
-    <t>mst_instructions4</t>
-  </si>
-  <si>
     <t>task_name</t>
   </si>
   <si>
-    <t>Melody Singing Task</t>
-  </si>
-  <si>
     <t>Please read the instructions carefully.</t>
   </si>
   <si>
@@ -123,6 +93,36 @@
   </si>
   <si>
     <t>In this task we’ll ask you to sing back a few notes and melodies that we play to you. It is fine if you think you are not a good singer. Throughout this first singing test, you will probably find some examples easy and others harder, and in general, as this specific singing test progresses, the trials become more challenging. Just always make your best attempt.</t>
+  </si>
+  <si>
+    <t>Welcome to the Singing Ability Assessment!</t>
+  </si>
+  <si>
+    <t>Singing Ability Assessment</t>
+  </si>
+  <si>
+    <t>SAA_welcome</t>
+  </si>
+  <si>
+    <t>SAA_welcome_1</t>
+  </si>
+  <si>
+    <t>SAA_welcome_2</t>
+  </si>
+  <si>
+    <t>SAA_instructions1</t>
+  </si>
+  <si>
+    <t>SAA_instructions2</t>
+  </si>
+  <si>
+    <t>SAA_instructions3</t>
+  </si>
+  <si>
+    <t>SAA_instructions4</t>
+  </si>
+  <si>
+    <t>SAA_button_play_note_and_sing</t>
   </si>
 </sst>
 </file>
@@ -548,79 +548,79 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>3</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="10" t="s">
-        <v>12</v>
+        <v>29</v>
       </c>
       <c r="B11" s="8" t="s">
         <v>0</v>
@@ -628,34 +628,34 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Add progress indicator feature
</commit_message>
<xml_diff>
--- a/data-raw/SAA.xlsx
+++ b/data-raw/SAA.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10111"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10313"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebsilas/Downloads/retranslations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebsilas/SAA/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{715ECFD8-67F5-EA49-8B74-C48B9B7643A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C48C48-96F5-B14A-AF12-69F6160C16A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="220" yWindow="1260" windowWidth="28800" windowHeight="17540" xr2:uid="{F918617E-B214-614F-96D8-792A3F23E788}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>In this task we’ll ask you to sing back a few notes and melodies that we play to you. It is fine if you think you are not a good singer. Throughout this first singing test, you will probably find some examples easy and others harder, and in general, as this specific singing test progresses, the trials become more challenging. Just always make your best attempt.</t>
   </si>
   <si>
-    <t>Welcome to the Singing Ability Assessment!</t>
-  </si>
-  <si>
     <t>Singing Ability Assessment</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
   </si>
   <si>
     <t>Wie Sie Singen sollten</t>
+  </si>
+  <si>
+    <t>Welcome to the</t>
   </si>
 </sst>
 </file>
@@ -567,97 +567,97 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="9" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>29</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="9" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="8" t="s">
         <v>0</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -668,7 +668,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -676,10 +676,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -690,7 +690,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -698,10 +698,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>